<commit_message>
Refine shoes transformer export behavior
</commit_message>
<xml_diff>
--- a/商品导入模板.xlsx
+++ b/商品导入模板.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29930"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6982FFCB-84B5-4628-A17A-B565F19AD704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28260" windowHeight="12600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="28260" windowHeight="12600"/>
   </bookViews>
   <sheets>
     <sheet name="商品信息" sheetId="4" r:id="rId1"/>
     <sheet name="计量单位" sheetId="5" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -32,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="157">
   <si>
     <t>空：默认根据标题生成</t>
   </si>
@@ -360,9 +356,6 @@
     <t>同一分类类目的商品填写相同售价（批量上传时填写）</t>
   </si>
   <si>
-    <t>随便填写，可统一设一个数字：99</t>
-  </si>
-  <si>
     <t>Air Jordan 1 Low GS 'Black Summit White' 553560-045</t>
   </si>
   <si>
@@ -374,7 +367,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>&lt;div class="tab-content tab-description rich-text" style="max-height: initial;" tab-first=""&gt;&lt;p&gt;Name:A</t>
+      <t>&lt;div class="tab-content tab-description rich-text" style="max-height: initial;" tab-first=""&gt;&lt;p&gt;Name:</t>
     </r>
     <r>
       <rPr>
@@ -384,27 +377,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>ir Jordan 1 Low GS 'Black Summit White'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;br&gt;Style:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>553560-045</t>
+      <t>Air Jordan 1 Low GS 'Black Summit White'553560-045</t>
     </r>
     <r>
       <rPr>
@@ -726,8 +699,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -758,6 +737,150 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="宋体"/>
@@ -772,7 +895,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -787,7 +910,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39994506668294322"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -809,8 +932,188 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -870,9 +1173,251 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -895,12 +1440,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -946,30 +1503,62 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1227,20 +1816,20 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:AG22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.899999999999999"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="3" width="18.375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="50.125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="50.1442307692308" style="4" customWidth="1"/>
     <col min="5" max="5" width="14.375" style="4" customWidth="1"/>
     <col min="6" max="6" width="51.25" style="4" customWidth="1"/>
-    <col min="7" max="7" width="36.75" style="4" customWidth="1"/>
+    <col min="7" max="7" width="36.7692307692308" style="4" customWidth="1"/>
     <col min="8" max="8" width="24" style="4" customWidth="1"/>
     <col min="9" max="9" width="12.75" style="4" customWidth="1"/>
     <col min="10" max="10" width="12" style="4" customWidth="1"/>
@@ -1257,7 +1846,7 @@
     <col min="24" max="24" width="93.75" style="4" customWidth="1"/>
     <col min="25" max="25" width="12.25" style="4" customWidth="1"/>
     <col min="26" max="27" width="15.5" style="4" customWidth="1"/>
-    <col min="28" max="28" width="40" style="4" customWidth="1"/>
+    <col min="28" max="28" width="39.9615384615385" style="4" customWidth="1"/>
     <col min="29" max="29" width="21" style="4" customWidth="1"/>
     <col min="30" max="30" width="12.5" style="4" customWidth="1"/>
     <col min="31" max="31" width="12.375" style="4" customWidth="1"/>
@@ -1266,234 +1855,234 @@
     <col min="34" max="16384" width="9" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="66" customHeight="1">
+    <row r="1" ht="66" customHeight="1" spans="1:33">
       <c r="W1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="X1" s="23" t="s">
+      <c r="X1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="24"/>
-      <c r="Z1" s="24"/>
-      <c r="AA1" s="25"/>
-      <c r="AB1" s="6" t="s">
+      <c r="Y1" s="7"/>
+      <c r="Z1" s="7"/>
+      <c r="AA1" s="8"/>
+      <c r="AB1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AC1" s="7"/>
-      <c r="AD1" s="26" t="s">
+      <c r="AC1" s="10"/>
+      <c r="AD1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="26"/>
-      <c r="AF1" s="26" t="s">
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="AG1" s="26"/>
-    </row>
-    <row r="2" spans="1:33" ht="17.100000000000001">
-      <c r="A2" s="8" t="s">
+      <c r="AG1" s="11"/>
+    </row>
+    <row r="2" ht="17" spans="1:33">
+      <c r="A2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="M2" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="9" t="s">
+      <c r="N2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="Q2" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="9" t="s">
+      <c r="R2" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="S2" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="T2" s="9" t="s">
+      <c r="T2" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="U2" s="9" t="s">
+      <c r="U2" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="V2" s="9" t="s">
+      <c r="V2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="W2" s="9" t="s">
+      <c r="W2" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="X2" s="10" t="s">
+      <c r="X2" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="Y2" s="10" t="s">
+      <c r="Y2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="Z2" s="10" t="s">
+      <c r="Z2" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="AA2" s="10" t="s">
+      <c r="AA2" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="AB2" s="10" t="s">
+      <c r="AB2" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="AC2" s="10" t="s">
+      <c r="AC2" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="AD2" s="11" t="s">
+      <c r="AD2" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="AE2" s="11" t="s">
+      <c r="AE2" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="AF2" s="11" t="s">
+      <c r="AF2" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="AG2" s="11" t="s">
+      <c r="AG2" s="15" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:33" s="1" customFormat="1" ht="68.099999999999994">
-      <c r="A3" s="8" t="s">
+    <row r="3" s="1" customFormat="1" ht="68" spans="1:33">
+      <c r="A3" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="J3" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="K3" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="L3" s="12" t="s">
+      <c r="L3" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="M3" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="N3" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="P3" s="12" t="s">
+      <c r="P3" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="Q3" s="12" t="s">
+      <c r="Q3" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="R3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="S3" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="T3" s="12" t="s">
+      <c r="T3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="U3" s="12" t="s">
+      <c r="U3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="V3" s="12" t="s">
+      <c r="V3" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="W3" s="12" t="s">
+      <c r="W3" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="X3" s="12" t="s">
+      <c r="X3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="Y3" s="12" t="s">
+      <c r="Y3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="Z3" s="12" t="s">
+      <c r="Z3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="AA3" s="12" t="s">
+      <c r="AA3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="AB3" s="12"/>
-      <c r="AC3" s="12" t="s">
+      <c r="AB3" s="16"/>
+      <c r="AC3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="AD3" s="12" t="s">
+      <c r="AD3" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="AE3" s="12" t="s">
+      <c r="AE3" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="AF3" s="12" t="s">
+      <c r="AF3" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="AG3" s="12" t="s">
+      <c r="AG3" s="16" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:33" s="2" customFormat="1" ht="135">
-      <c r="A4" s="13" t="s">
+    <row r="4" s="2" customFormat="1" ht="185" spans="1:33">
+      <c r="A4" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="17" t="s">
         <v>62</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1584,267 +2173,231 @@
         <v>63</v>
       </c>
       <c r="AF4" s="2" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="AG4" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:33" s="3" customFormat="1" ht="320.10000000000002">
-      <c r="B5" s="14" t="s">
+    <row r="5" s="3" customFormat="1" ht="320" spans="1:33">
+      <c r="B5" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="19"/>
+      <c r="D5" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="16" t="s">
+      <c r="E5" t="s">
         <v>83</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="G5" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="H5" s="21"/>
+      <c r="I5" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="H5" s="17"/>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="J5" s="15" t="s">
+      <c r="L5" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="L5" s="16" t="s">
+      <c r="M5" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="M5" s="18" t="s">
+      <c r="N5" s="19"/>
+      <c r="O5" s="19" t="s">
         <v>90</v>
-      </c>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15" t="s">
-        <v>91</v>
       </c>
       <c r="P5" s="3">
         <v>2</v>
       </c>
-      <c r="T5" s="16" t="s">
+      <c r="T5" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="U5" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="U5" s="16" t="s">
+      <c r="V5" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="V5" s="17" t="s">
+      <c r="W5" s="20"/>
+      <c r="X5" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="W5" s="16"/>
-      <c r="X5" s="16" t="s">
+      <c r="Y5" s="20"/>
+      <c r="Z5" s="19"/>
+      <c r="AA5" s="19"/>
+      <c r="AB5" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="Y5" s="16"/>
-      <c r="Z5" s="15"/>
-      <c r="AA5" s="15"/>
-      <c r="AB5" s="16" t="s">
-        <v>96</v>
-      </c>
+      <c r="AC5" s="3"/>
       <c r="AD5" s="3">
         <v>99</v>
       </c>
-      <c r="AF5" s="3">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:33" ht="15.95" customHeight="1">
-      <c r="D6" s="19"/>
-      <c r="X6" s="20"/>
+    </row>
+    <row r="6" ht="16" customHeight="1" spans="1:33">
+      <c r="D6" s="23"/>
+      <c r="X6" s="24"/>
       <c r="Z6" s="1"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="AC6" s="21"/>
+      <c r="AB6" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="AC6" s="25"/>
       <c r="AD6" s="3">
         <v>99</v>
       </c>
-      <c r="AE6" s="22"/>
-      <c r="AF6" s="3">
-        <v>99</v>
-      </c>
+      <c r="AE6" s="26"/>
+      <c r="AF6" s="3"/>
     </row>
     <row r="7" spans="1:33">
       <c r="AB7" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AD7" s="3">
         <v>99</v>
       </c>
-      <c r="AF7" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF7" s="3"/>
     </row>
     <row r="8" spans="1:33">
       <c r="AB8" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AD8" s="3">
         <v>99</v>
       </c>
-      <c r="AF8" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF8" s="3"/>
     </row>
     <row r="9" spans="1:33">
       <c r="AB9" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AD9" s="3">
         <v>99</v>
       </c>
-      <c r="AF9" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF9" s="3"/>
     </row>
     <row r="10" spans="1:33">
       <c r="AB10" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AD10" s="3">
         <v>99</v>
       </c>
-      <c r="AF10" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF10" s="3"/>
     </row>
     <row r="11" spans="1:33">
       <c r="AB11" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AD11" s="3">
         <v>99</v>
       </c>
-      <c r="AF11" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF11" s="3"/>
     </row>
     <row r="12" spans="1:33">
       <c r="AB12" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AD12" s="3">
         <v>99</v>
       </c>
-      <c r="AF12" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF12" s="3"/>
     </row>
     <row r="13" spans="1:33">
       <c r="AB13" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AD13" s="3">
         <v>99</v>
       </c>
-      <c r="AF13" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF13" s="3"/>
     </row>
     <row r="14" spans="1:33">
       <c r="AB14" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AD14" s="3">
         <v>99</v>
       </c>
-      <c r="AF14" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF14" s="3"/>
     </row>
     <row r="15" spans="1:33">
       <c r="AB15" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="AD15" s="3">
         <v>99</v>
       </c>
-      <c r="AF15" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF15" s="3"/>
     </row>
     <row r="16" spans="1:33">
       <c r="AB16" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AD16" s="3">
         <v>99</v>
       </c>
-      <c r="AF16" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF16" s="3"/>
     </row>
     <row r="17" spans="28:32">
       <c r="AB17" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD17" s="3">
         <v>99</v>
       </c>
-      <c r="AF17" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF17" s="3"/>
     </row>
     <row r="18" spans="28:32">
       <c r="AB18" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AD18" s="3">
         <v>99</v>
       </c>
-      <c r="AF18" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF18" s="3"/>
     </row>
     <row r="19" spans="28:32">
       <c r="AB19" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AD19" s="3">
         <v>99</v>
       </c>
-      <c r="AF19" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF19" s="3"/>
     </row>
     <row r="20" spans="28:32">
       <c r="AB20" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AD20" s="3">
         <v>99</v>
       </c>
-      <c r="AF20" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF20" s="3"/>
     </row>
     <row r="21" spans="28:32">
       <c r="AB21" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="AD21" s="3">
         <v>99</v>
       </c>
-      <c r="AF21" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF21" s="3"/>
     </row>
     <row r="22" spans="28:32">
       <c r="AB22" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AD22" s="3">
         <v>99</v>
       </c>
-      <c r="AF22" s="3">
-        <v>99</v>
-      </c>
+      <c r="AF22" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1852,245 +2405,248 @@
     <mergeCell ref="AD1:AE1"/>
     <mergeCell ref="AF1:AG1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555596" footer="0.51180555555555596"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
   <pageSetup paperSize="9" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:A45"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.899999999999999"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="18.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update import template prices
</commit_message>
<xml_diff>
--- a/商品导入模板.xlsx
+++ b/商品导入模板.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11210"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/a1-6/Desktop/work/commerce-tool/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9362F98A-FAD8-9F49-96EF-F84BAB62F9C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="28260" windowHeight="12600"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="商品信息" sheetId="4" r:id="rId1"/>
@@ -19,7 +25,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -699,14 +704,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -734,151 +733,7 @@
       <sz val="9"/>
       <color rgb="FF202124"/>
       <name val="Consolas"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -894,8 +749,15 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="37">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -910,7 +772,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.39994506668294322"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -932,188 +794,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="13">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1173,259 +855,17 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1434,29 +874,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1470,21 +895,12 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1492,9 +908,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
@@ -1503,62 +916,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1816,273 +1197,273 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AG22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="3" width="18.375" style="4" customWidth="1"/>
-    <col min="4" max="4" width="50.1442307692308" style="4" customWidth="1"/>
-    <col min="5" max="5" width="14.375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="51.25" style="4" customWidth="1"/>
-    <col min="7" max="7" width="36.7692307692308" style="4" customWidth="1"/>
-    <col min="8" max="8" width="24" style="4" customWidth="1"/>
-    <col min="9" max="9" width="12.75" style="4" customWidth="1"/>
-    <col min="10" max="10" width="12" style="4" customWidth="1"/>
-    <col min="11" max="11" width="15.75" style="4" customWidth="1"/>
-    <col min="12" max="13" width="15.375" style="4" customWidth="1"/>
-    <col min="14" max="15" width="15.25" style="4" customWidth="1"/>
-    <col min="16" max="16" width="13" style="4" customWidth="1"/>
-    <col min="17" max="17" width="13.125" style="4" customWidth="1"/>
-    <col min="18" max="19" width="11.75" style="4" customWidth="1"/>
-    <col min="20" max="20" width="16" style="4" customWidth="1"/>
-    <col min="21" max="21" width="14.875" style="4" customWidth="1"/>
-    <col min="22" max="22" width="16" style="4" customWidth="1"/>
-    <col min="23" max="23" width="22.375" style="4" customWidth="1"/>
-    <col min="24" max="24" width="93.75" style="4" customWidth="1"/>
-    <col min="25" max="25" width="12.25" style="4" customWidth="1"/>
-    <col min="26" max="27" width="15.5" style="4" customWidth="1"/>
-    <col min="28" max="28" width="39.9615384615385" style="4" customWidth="1"/>
-    <col min="29" max="29" width="21" style="4" customWidth="1"/>
-    <col min="30" max="30" width="12.5" style="4" customWidth="1"/>
-    <col min="31" max="31" width="12.375" style="4" customWidth="1"/>
-    <col min="32" max="32" width="9.75" style="4" customWidth="1"/>
-    <col min="33" max="33" width="13.375" style="4" customWidth="1"/>
-    <col min="34" max="16384" width="9" style="4"/>
+    <col min="1" max="3" width="18.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="50.1640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="51.1640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="36.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="24" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.6640625" style="1" customWidth="1"/>
+    <col min="12" max="13" width="15.33203125" style="1" customWidth="1"/>
+    <col min="14" max="15" width="15.1640625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="13" style="1" customWidth="1"/>
+    <col min="17" max="17" width="13.1640625" style="1" customWidth="1"/>
+    <col min="18" max="19" width="11.6640625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="16" style="1" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" style="1" customWidth="1"/>
+    <col min="22" max="22" width="16" style="1" customWidth="1"/>
+    <col min="23" max="23" width="22.33203125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="93.6640625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="12.1640625" style="1" customWidth="1"/>
+    <col min="26" max="27" width="15.5" style="1" customWidth="1"/>
+    <col min="28" max="28" width="40" style="1" customWidth="1"/>
+    <col min="29" max="29" width="21" style="1" customWidth="1"/>
+    <col min="30" max="30" width="12.5" style="1" customWidth="1"/>
+    <col min="31" max="31" width="12.33203125" style="1" customWidth="1"/>
+    <col min="32" max="32" width="9.6640625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="13.33203125" style="1" customWidth="1"/>
+    <col min="34" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="66" customHeight="1" spans="1:33">
-      <c r="W1" s="5" t="s">
+    <row r="1" spans="1:33" ht="66" customHeight="1">
+      <c r="W1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="X1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="7"/>
-      <c r="Z1" s="7"/>
-      <c r="AA1" s="8"/>
-      <c r="AB1" s="9" t="s">
+      <c r="Y1" s="19"/>
+      <c r="Z1" s="19"/>
+      <c r="AA1" s="20"/>
+      <c r="AB1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="AC1" s="10"/>
-      <c r="AD1" s="11" t="s">
+      <c r="AC1" s="6"/>
+      <c r="AD1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="11"/>
-      <c r="AF1" s="11" t="s">
+      <c r="AE1" s="21"/>
+      <c r="AF1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="AG1" s="11"/>
-    </row>
-    <row r="2" ht="17" spans="1:33">
-      <c r="A2" s="12" t="s">
+      <c r="AG1" s="21"/>
+    </row>
+    <row r="2" spans="1:33" ht="15">
+      <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="L2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="N2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="R2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="S2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="T2" s="13" t="s">
+      <c r="T2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="U2" s="13" t="s">
+      <c r="U2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="V2" s="13" t="s">
+      <c r="V2" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="W2" s="13" t="s">
+      <c r="W2" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="X2" s="14" t="s">
+      <c r="X2" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="Y2" s="14" t="s">
+      <c r="Y2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="Z2" s="14" t="s">
+      <c r="Z2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="AA2" s="14" t="s">
+      <c r="AA2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="AB2" s="14" t="s">
+      <c r="AB2" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="AC2" s="14" t="s">
+      <c r="AC2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="AD2" s="15" t="s">
+      <c r="AD2" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="AE2" s="15" t="s">
+      <c r="AE2" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="AF2" s="15" t="s">
+      <c r="AF2" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="AG2" s="15" t="s">
+      <c r="AG2" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" ht="68" spans="1:33">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:33" ht="60">
+      <c r="A3" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="J3" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="L3" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="M3" s="16" t="s">
+      <c r="M3" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="N3" s="16" t="s">
+      <c r="N3" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="O3" s="16" t="s">
+      <c r="O3" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="P3" s="16" t="s">
+      <c r="P3" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="Q3" s="16" t="s">
+      <c r="Q3" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="R3" s="16" t="s">
+      <c r="R3" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="S3" s="16" t="s">
+      <c r="S3" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="T3" s="16" t="s">
+      <c r="T3" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="U3" s="16" t="s">
+      <c r="U3" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="V3" s="16" t="s">
+      <c r="V3" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="W3" s="16" t="s">
+      <c r="W3" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="X3" s="16" t="s">
+      <c r="X3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="Y3" s="16" t="s">
+      <c r="Y3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="Z3" s="16" t="s">
+      <c r="Z3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="AA3" s="16" t="s">
+      <c r="AA3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="AB3" s="16"/>
-      <c r="AC3" s="16" t="s">
+      <c r="AB3" s="11"/>
+      <c r="AC3" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="AD3" s="16" t="s">
+      <c r="AD3" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="AE3" s="16" t="s">
+      <c r="AE3" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="AF3" s="16" t="s">
+      <c r="AF3" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="AG3" s="16" t="s">
+      <c r="AG3" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" s="2" customFormat="1" ht="185" spans="1:33">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:33" s="2" customFormat="1" ht="150">
+      <c r="A4" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -2179,223 +1560,216 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" s="3" customFormat="1" ht="320" spans="1:33">
-      <c r="B5" s="18" t="s">
+    <row r="5" spans="1:33" s="3" customFormat="1" ht="285">
+      <c r="B5" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="13" t="s">
         <v>82</v>
       </c>
       <c r="E5" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="H5" s="21"/>
+      <c r="H5" s="13"/>
       <c r="I5" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="M5" s="22" t="s">
+      <c r="M5" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19" t="s">
+      <c r="O5" s="3" t="s">
         <v>90</v>
       </c>
       <c r="P5" s="3">
         <v>2</v>
       </c>
-      <c r="T5" s="20" t="s">
+      <c r="T5" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="U5" s="20" t="s">
+      <c r="U5" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="V5" s="21" t="s">
+      <c r="V5" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="W5" s="20"/>
-      <c r="X5" s="20" t="s">
+      <c r="W5" s="13"/>
+      <c r="X5" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="Y5" s="20"/>
-      <c r="Z5" s="19"/>
-      <c r="AA5" s="19"/>
-      <c r="AB5" s="20" t="s">
+      <c r="Y5" s="13"/>
+      <c r="AB5" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="AC5" s="3"/>
       <c r="AD5" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" ht="16" customHeight="1">
+      <c r="D6" s="4"/>
+      <c r="X6" s="15"/>
+      <c r="AB6" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="AC6" s="16"/>
+      <c r="AD6" s="3">
+        <v>100</v>
+      </c>
+      <c r="AE6" s="17"/>
+      <c r="AF6" s="3"/>
+    </row>
+    <row r="7" spans="1:33">
+      <c r="AB7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AD7" s="3">
+        <v>100</v>
+      </c>
+      <c r="AF7" s="3"/>
+    </row>
+    <row r="8" spans="1:33">
+      <c r="AB8" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="AD8" s="3">
+        <v>100</v>
+      </c>
+      <c r="AF8" s="3"/>
+    </row>
+    <row r="9" spans="1:33">
+      <c r="AB9" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="6" ht="16" customHeight="1" spans="1:33">
-      <c r="D6" s="23"/>
-      <c r="X6" s="24"/>
-      <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-      <c r="AB6" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="AC6" s="25"/>
-      <c r="AD6" s="3">
-        <v>99</v>
-      </c>
-      <c r="AE6" s="26"/>
-      <c r="AF6" s="3"/>
-    </row>
-    <row r="7" spans="1:33">
-      <c r="AB7" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="AD7" s="3">
-        <v>99</v>
-      </c>
-      <c r="AF7" s="3"/>
-    </row>
-    <row r="8" spans="1:33">
-      <c r="AB8" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="AD8" s="3">
-        <v>99</v>
-      </c>
-      <c r="AF8" s="3"/>
-    </row>
-    <row r="9" spans="1:33">
-      <c r="AB9" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="AD9" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF9" s="3"/>
     </row>
     <row r="10" spans="1:33">
-      <c r="AB10" s="4" t="s">
+      <c r="AB10" s="1" t="s">
         <v>100</v>
       </c>
       <c r="AD10" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF10" s="3"/>
     </row>
     <row r="11" spans="1:33">
-      <c r="AB11" s="4" t="s">
+      <c r="AB11" s="1" t="s">
         <v>101</v>
       </c>
       <c r="AD11" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF11" s="3"/>
     </row>
     <row r="12" spans="1:33">
-      <c r="AB12" s="4" t="s">
+      <c r="AB12" s="1" t="s">
         <v>102</v>
       </c>
       <c r="AD12" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF12" s="3"/>
     </row>
     <row r="13" spans="1:33">
-      <c r="AB13" s="4" t="s">
+      <c r="AB13" s="1" t="s">
         <v>103</v>
       </c>
       <c r="AD13" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF13" s="3"/>
     </row>
     <row r="14" spans="1:33">
-      <c r="AB14" s="4" t="s">
+      <c r="AB14" s="1" t="s">
         <v>104</v>
       </c>
       <c r="AD14" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF14" s="3"/>
     </row>
     <row r="15" spans="1:33">
-      <c r="AB15" s="4" t="s">
+      <c r="AB15" s="1" t="s">
         <v>105</v>
       </c>
       <c r="AD15" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF15" s="3"/>
     </row>
     <row r="16" spans="1:33">
-      <c r="AB16" s="4" t="s">
+      <c r="AB16" s="1" t="s">
         <v>106</v>
       </c>
       <c r="AD16" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF16" s="3"/>
     </row>
     <row r="17" spans="28:32">
-      <c r="AB17" s="4" t="s">
+      <c r="AB17" s="1" t="s">
         <v>107</v>
       </c>
       <c r="AD17" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF17" s="3"/>
     </row>
     <row r="18" spans="28:32">
-      <c r="AB18" s="4" t="s">
+      <c r="AB18" s="1" t="s">
         <v>108</v>
       </c>
       <c r="AD18" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF18" s="3"/>
     </row>
     <row r="19" spans="28:32">
-      <c r="AB19" s="4" t="s">
+      <c r="AB19" s="1" t="s">
         <v>109</v>
       </c>
       <c r="AD19" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF19" s="3"/>
     </row>
     <row r="20" spans="28:32">
-      <c r="AB20" s="4" t="s">
+      <c r="AB20" s="1" t="s">
         <v>110</v>
       </c>
       <c r="AD20" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF20" s="3"/>
     </row>
     <row r="21" spans="28:32">
-      <c r="AB21" s="4" t="s">
+      <c r="AB21" s="1" t="s">
         <v>111</v>
       </c>
       <c r="AD21" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF21" s="3"/>
     </row>
     <row r="22" spans="28:32">
-      <c r="AB22" s="4" t="s">
+      <c r="AB22" s="1" t="s">
         <v>112</v>
       </c>
       <c r="AD22" s="3">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AF22" s="3"/>
     </row>
@@ -2405,19 +1779,18 @@
     <mergeCell ref="AD1:AE1"/>
     <mergeCell ref="AF1:AG1"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555556" footer="0.511805555555556"/>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555596" footer="0.51180555555555596"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A45"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="18.625" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -2646,7 +2019,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>